<commit_message>
S2a — Layer 1b: FAA NOTAM API source (tier-1 hubs, 23 airports). Adds international NOTAM coverage via FAA External NOTAM API — highest-quality free NOTAM source we can use (global, not just US airspace, stable JSON schema, no scraping). Fetches per-airport for airports.TIER1_ICAO on nightly cron; tier-2 airports remain queryable on-demand by the app but not pulled nightly to keep well under the rate limit. Per-NOTAM payload trimmed to core fields: id, number, type, classification, series, location, effective_start/end, text. Requires free registration at https://api.faa.gov/s/ then FAA_CLIENT_ID + FAA_CLIENT_SECRET as GitHub Actions secrets — until secrets set, module raises actionable RuntimeError which the runner captures into the manifest Notes column. Manifest register updated (11 sources total).
</commit_message>
<xml_diff>
--- a/data/manifest.xlsx
+++ b/data/manifest.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +29,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="13"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,17 +56,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,15 +429,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -924,22 +915,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>vaac-london-qva</t>
+          <t>faa-notams</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Volcanic ash</t>
+          <t>NOTAMs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Met Office VAAC London</t>
+          <t>FAA External NOTAM API</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>QVA@metoffice.gov.uk</t>
+          <t>https://external-api.faa.gov/notamapi/v1/notams</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -949,7 +940,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>written request</t>
+          <t>clientId + clientSecret</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -959,7 +950,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L1b</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -973,85 +964,175 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>DefendAble — evidence-collection · manifest.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Live register of every data source. One row per source. Updated in place by the nightly cron (run_all.py).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Do not edit Source ID / Category / Provider / Endpoint / Cadence / Auth / Cost / Layer / Notes by hand — those come from manifest_source_of_truth.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Status / Last pull / Rows / Bytes / Live URL are overwritten each run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Status values: planned (not yet implemented) · live (successful last run) · failed (last run errored — see [last error …] prefix in Notes).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Layers: L1 free · L2 paid single-fee · L3 usage-billed.</t>
+          <t>International NOTAM coverage — tier-1 hubs only for nightly pull; on-demand for tier-2. Needs free FAA_CLIENT_ID + FAA_CLIENT_SECRET secrets.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>aviation-herald-news</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>The Aviation Herald</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://avherald.com/h?rss.php</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>L1b</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Incident-focused aviation news — every serious event within 24-48h. Practitioner-standard.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>See README.md at repo root for the full pipeline overview.</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>simple-flying-news</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Simple Flying</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://simpleflying.com/feed/</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>L1b</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Broader aviation news + regulatory + operational context. Tagged by category on pull.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>vaac-london-qva</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Volcanic ash</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Met Office VAAC London</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>QVA@metoffice.gov.uk</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>written request</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S2d — Layer 1b: GDACS global disaster alerts. Adds the UN + EU joint natural-disaster feed — earthquakes / tropical cyclones / floods / volcanoes / droughts / wildfires. Every event carries a GDACS-scored alert level (Green / Orange / Red) that lets the UI colour-code impact severity. Free JSON, no auth, no rate limit. Per-event payload: id, type, name, country, iso3, alert_level, alert_score, severity, affected population, from/to date, report URL, lat/lon. Includes by_type + by_alert_level roll-ups for dashboard KPI use. This is the source that catches cases like 'Turkish earthquake grounded flights out of IST' before we know to look.
</commit_message>
<xml_diff>
--- a/data/manifest.xlsx
+++ b/data/manifest.xlsx
@@ -429,12 +429,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -1083,22 +1083,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>vaac-london-qva</t>
+          <t>gdacs-global-disasters</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Volcanic ash</t>
+          <t>Natural disaster</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Met Office VAAC London</t>
+          <t>GDACS (UN + EU)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>QVA@metoffice.gov.uk</t>
+          <t>https://www.gdacs.org/gdacsapi/api/events/geteventlist/EVENTS</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>written request</t>
+          <t>none</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L1b</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1132,6 +1132,230 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
+          <t>Global disasters — earthquakes / floods / storms / volcanoes / droughts / wildfires. UN + EU joint feed. Severity-scored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>smithsonian-volcanoes</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Volcanic activity</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Smithsonian Global Volcanism Program</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://volcano.si.edu/news/WeeklyVolcanoRSS.xml</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>L1b</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Weekly report of currently-erupting or recently-active volcanoes. Upstream of VAAC ash advisories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>met-office-charts</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>UK Met Office</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.metoffice.gov.uk/services/transport/aviation/regulated/general-aviation</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>L1b</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Aviation weather charts (MSLP / F214 / F215 / sig-wx). URLs stored; images lazy-loaded by UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>eurocontrol-coda</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ATFM</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Eurocontrol CODA</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eurocontrol.int/publications</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>L1b</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Central Office for Delay Analysis publications — retrospective ATFM delay stats. Companion to live NM feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>vaac-london-qva</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Volcanic ash</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Met Office VAAC London</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>QVA@metoffice.gov.uk</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>written request</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
           <t>QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
         </is>
       </c>

</xml_diff>

<commit_message>
S3 — retention job (90-day full + monthly rollups). New retention.py implements the retention policy: any snapshot in data/YYYY-MM-DD/ older than 90 days is archived into data/rollup/YYYY-MM/<source-id>.json as an append-only list of {date, pulled_at, rows, endpoint, first_item, archived_bytes} entries — one per original file. Original dated snapshot is then deleted and the empty date directory removed. Idempotent, stdlib-only, safe to re-run. Wired into run_all.py as final step after every nightly run (after append_log) — prints archive stats to stdout so GitHub Actions logs show what got rolled up. Rationale: as we scale up to 15+ sources at ~50KB each per day, unbounded retention grows the repo ~30MB/mo. Rollups preserve searchability for older cases (date + pulled_at + rows + endpoint + first-item summary still queryable) while capping repo growth. First rollup will fire ~90 days after the first live pull; until then this is a no-op. Test suite unaffected.
</commit_message>
<xml_diff>
--- a/data/manifest.xlsx
+++ b/data/manifest.xlsx
@@ -563,16 +563,24 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>METAR + TAF for named-airport list — Ogimet replacement</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · METAR + TAF for named-airport list — Ogimet replacement</t>
         </is>
       </c>
     </row>
@@ -619,16 +627,24 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>ADS-B flight tracks — TOPS replacement for basic coverage</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · ADS-B flight tracks — TOPS replacement for basic coverage</t>
         </is>
       </c>
     </row>
@@ -675,16 +691,24 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Active wildfire hotspots — natural-disaster evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: FIRMS_MAP_KEY env var missing — register free key at https://firms.modaps.eosdis.nasa.gov/api/map_key/ and add to GitHub Actions secrets. · Active wildfire hotspots — natural-disaster evidence</t>
         </is>
       </c>
     </row>
@@ -731,16 +755,24 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>EU forest-fire snapshots — natural-disaster evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · EU forest-fire snapshots — natural-disaster evidence</t>
         </is>
       </c>
     </row>
@@ -787,16 +819,24 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>French ATC industrial-action notices — third-party IA evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · French ATC industrial-action notices — third-party IA evidence</t>
         </is>
       </c>
     </row>
@@ -843,16 +883,24 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Italian aviation industrial-action notices — third-party IA evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Italian aviation industrial-action notices — third-party IA evidence</t>
         </is>
       </c>
     </row>
@@ -899,16 +947,24 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Public NM regulations feed — ATFM cascade evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Public NM regulations feed — ATFM cascade evidence</t>
         </is>
       </c>
     </row>
@@ -955,16 +1011,24 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>International NOTAM coverage — tier-1 hubs only for nightly pull; on-demand for tier-2. Needs free FAA_CLIENT_ID + FAA_CLIENT_SECRET secrets.</t>
+          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: FAA_CLIENT_ID / FAA_CLIENT_SECRET env vars missing — register free at https://api.faa.gov/s/ and add as GitHub Actions secrets. · International NOTAM coverage — tier-1 hubs only for nightly pull; on-demand for tier-2. Needs free FAA_CLIENT_ID + FAA_CLIENT_SECRET secrets.</t>
         </is>
       </c>
     </row>
@@ -1011,16 +1075,24 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Incident-focused aviation news — every serious event within 24-48h. Practitioner-standard.</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Incident-focused aviation news — every serious event within 24-48h. Practitioner-standard.</t>
         </is>
       </c>
     </row>
@@ -1067,16 +1139,24 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Broader aviation news + regulatory + operational context. Tagged by category on pull.</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Broader aviation news + regulatory + operational context. Tagged by category on pull.</t>
         </is>
       </c>
     </row>
@@ -1123,16 +1203,24 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Global disasters — earthquakes / floods / storms / volcanoes / droughts / wildfires. UN + EU joint feed. Severity-scored.</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Global disasters — earthquakes / floods / storms / volcanoes / droughts / wildfires. UN + EU joint feed. Severity-scored.</t>
         </is>
       </c>
     </row>
@@ -1179,16 +1267,24 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Weekly report of currently-erupting or recently-active volcanoes. Upstream of VAAC ash advisories.</t>
+          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Weekly report of currently-erupting or recently-active volcanoes. Upstream of VAAC ash advisories.</t>
         </is>
       </c>
     </row>
@@ -1235,13 +1331,25 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>1144</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/evansharry165-wq/evidence-collection/main/data/latest/met-office-charts.json</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Aviation weather charts (MSLP / F214 / F215 / sig-wx). URLs stored; images lazy-loaded by UI.</t>
@@ -1291,13 +1399,25 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="2" t="n">
+        <v>476</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/evansharry165-wq/evidence-collection/main/data/latest/eurocontrol-coda.json</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Central Office for Delay Analysis publications — retrospective ATFM delay stats. Companion to live NM feed.</t>
@@ -1347,16 +1467,24 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25T20:04:06Z</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
+          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: VAAC QVA access not yet onboarded — email QVA@metoffice.gov.uk with the subscription template in this file's docstring. Free but access-gated. · QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add source: AutoRouter European NOTAM feed (Layer 1b upgrade over FAA). AutoRouter.aero provides free-tier NOTAM coverage for European FIRs — materially better than the FAA NOTAM API (US-biased, current-only) that daily source has been our only NOTAM feed. Free registration at autorouter.aero → HTTP Basic auth via AUTOROUTER_USER + AUTOROUTER_PASS env-vars → GitHub Actions secrets. Pulls per-airport for TIER1_ICAO on nightly cron; same shape as faa-notams source. Per-NOTAM payload: id / series / number / type / issued / effective_start-end / location / traffic / purpose / scope / text plus raw for downstream inspection. Historical query (what was live at a specific past time — the shape case work actually needs) is a follow-up on-demand source that this daily module doesn't attempt. Manifest register updated (16 sources total).
</commit_message>
<xml_diff>
--- a/data/manifest.xlsx
+++ b/data/manifest.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -437,8 +437,8 @@
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -563,24 +563,16 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · METAR + TAF for named-airport list — Ogimet replacement</t>
+          <t>METAR + TAF for named-airport list — Ogimet replacement</t>
         </is>
       </c>
     </row>
@@ -627,24 +619,16 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · ADS-B flight tracks — TOPS replacement for basic coverage</t>
+          <t>ADS-B flight tracks — TOPS replacement for basic coverage</t>
         </is>
       </c>
     </row>
@@ -691,24 +675,16 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: FIRMS_MAP_KEY env var missing — register free key at https://firms.modaps.eosdis.nasa.gov/api/map_key/ and add to GitHub Actions secrets. · Active wildfire hotspots — natural-disaster evidence</t>
+          <t>Active wildfire hotspots — natural-disaster evidence</t>
         </is>
       </c>
     </row>
@@ -755,24 +731,16 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · EU forest-fire snapshots — natural-disaster evidence</t>
+          <t>EU forest-fire snapshots — natural-disaster evidence</t>
         </is>
       </c>
     </row>
@@ -819,24 +787,16 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · French ATC industrial-action notices — third-party IA evidence</t>
+          <t>French ATC industrial-action notices — third-party IA evidence</t>
         </is>
       </c>
     </row>
@@ -883,24 +843,16 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Italian aviation industrial-action notices — third-party IA evidence</t>
+          <t>Italian aviation industrial-action notices — third-party IA evidence</t>
         </is>
       </c>
     </row>
@@ -947,24 +899,16 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Public NM regulations feed — ATFM cascade evidence</t>
+          <t>Public NM regulations feed — ATFM cascade evidence</t>
         </is>
       </c>
     </row>
@@ -1011,24 +955,16 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: FAA_CLIENT_ID / FAA_CLIENT_SECRET env vars missing — register free at https://api.faa.gov/s/ and add as GitHub Actions secrets. · International NOTAM coverage — tier-1 hubs only for nightly pull; on-demand for tier-2. Needs free FAA_CLIENT_ID + FAA_CLIENT_SECRET secrets.</t>
+          <t>International NOTAM coverage — tier-1 hubs only for nightly pull; on-demand for tier-2. Needs free FAA_CLIENT_ID + FAA_CLIENT_SECRET secrets.</t>
         </is>
       </c>
     </row>
@@ -1075,24 +1011,16 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Incident-focused aviation news — every serious event within 24-48h. Practitioner-standard.</t>
+          <t>Incident-focused aviation news — every serious event within 24-48h. Practitioner-standard.</t>
         </is>
       </c>
     </row>
@@ -1139,24 +1067,16 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Broader aviation news + regulatory + operational context. Tagged by category on pull.</t>
+          <t>Broader aviation news + regulatory + operational context. Tagged by category on pull.</t>
         </is>
       </c>
     </row>
@@ -1203,24 +1123,16 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Global disasters — earthquakes / floods / storms / volcanoes / droughts / wildfires. UN + EU joint feed. Severity-scored.</t>
+          <t>Global disasters — earthquakes / floods / storms / volcanoes / droughts / wildfires. UN + EU joint feed. Severity-scored.</t>
         </is>
       </c>
     </row>
@@ -1267,24 +1179,16 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] URLError: &lt;urlopen error Tunnel connection failed: 403 Forbidden&gt; · Weekly report of currently-erupting or recently-active volcanoes. Upstream of VAAC ash advisories.</t>
+          <t>Weekly report of currently-erupting or recently-active volcanoes. Upstream of VAAC ash advisories.</t>
         </is>
       </c>
     </row>
@@ -1331,25 +1235,13 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>1144</v>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/evansharry165-wq/evidence-collection/main/data/latest/met-office-charts.json</t>
-        </is>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Aviation weather charts (MSLP / F214 / F215 / sig-wx). URLs stored; images lazy-loaded by UI.</t>
@@ -1399,25 +1291,13 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>476</v>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/evansharry165-wq/evidence-collection/main/data/latest/eurocontrol-coda.json</t>
-        </is>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Central Office for Delay Analysis publications — retrospective ATFM delay stats. Companion to live NM feed.</t>
@@ -1427,22 +1307,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>vaac-london-qva</t>
+          <t>autorouter-notams</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Volcanic ash</t>
+          <t>NOTAMs</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Met Office VAAC London</t>
+          <t>AutoRouter</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>QVA@metoffice.gov.uk</t>
+          <t>https://api.autorouter.aero/v1.0/notam</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1452,39 +1332,87 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>written request</t>
+          <t>HTTP Basic (AUTOROUTER_USER + AUTOROUTER_PASS)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>free (register)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L1b</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25T20:04:06Z</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>[last error 2026-07-25T20:04:06Z] RuntimeError: VAAC QVA access not yet onboarded — email QVA@metoffice.gov.uk with the subscription template in this file's docstring. Free but access-gated. · QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
+          <t>Better European coverage than FAA NOTAM (US-biased, current-only). Free tier. Historical query = follow-up on-demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>vaac-london-qva</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Volcanic ash</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Met Office VAAC London</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>QVA@metoffice.gov.uk</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>daily 03:00</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>written request</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>free</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>QVA quantitative volcanic-ash feed — McDonagh-style evidence</t>
         </is>
       </c>
     </row>

</xml_diff>